<commit_message>
docs: finalized test plan coverage metrics and presentation formatting after review
</commit_message>
<xml_diff>
--- a/Свод(чек-лист+тест-кейс+баг-репор+автоматизация)/Тестирование сайта Стейк'S Свод_документов.xlsx
+++ b/Свод(чек-лист+тест-кейс+баг-репор+автоматизация)/Тестирование сайта Стейк'S Свод_документов.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hidden\Desktop\Финальный проект_АКАДЕМИЯ ТОП\Мой_ДИПЛОМНЫЙ_ПРОЕКТ\Свод(чек-лист+тест-кейс+баг-репор+автоматизация)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3D64D26-D236-4C38-8440-38F1336B433B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{664B5402-3EA7-4BB6-B7BE-2AA0769C4157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Чек-лист" sheetId="1" r:id="rId1"/>
@@ -4314,10 +4314,26 @@
     <xf numFmtId="0" fontId="55" fillId="27" borderId="0" xfId="6" applyFill="1"/>
     <xf numFmtId="0" fontId="50" fillId="27" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="51" fillId="27" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4325,33 +4341,8 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -4362,17 +4353,26 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="39" fillId="19" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="38" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="39" fillId="3" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -13864,27 +13864,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="13.8">
-      <c r="A1" s="129" t="s">
+      <c r="A1" s="137" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="131" t="s">
+      <c r="B1" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="132"/>
-      <c r="D1" s="136" t="s">
+      <c r="C1" s="133"/>
+      <c r="D1" s="131" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="137"/>
-      <c r="F1" s="132"/>
-      <c r="G1" s="138" t="s">
+      <c r="E1" s="132"/>
+      <c r="F1" s="133"/>
+      <c r="G1" s="134" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="134" t="s">
+      <c r="H1" s="127" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="55.2">
-      <c r="A2" s="130"/>
+      <c r="A2" s="138"/>
       <c r="B2" s="23" t="s">
         <v>5</v>
       </c>
@@ -13900,11 +13900,11 @@
       <c r="F2" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="139"/>
-      <c r="H2" s="135"/>
+      <c r="G2" s="135"/>
+      <c r="H2" s="128"/>
     </row>
     <row r="3" spans="1:25" ht="13.8">
-      <c r="A3" s="133" t="s">
+      <c r="A3" s="129" t="s">
         <v>51</v>
       </c>
       <c r="B3" s="13" t="s">
@@ -13926,7 +13926,7 @@
       <c r="H3" s="16"/>
     </row>
     <row r="4" spans="1:25" ht="13.8">
-      <c r="A4" s="128"/>
+      <c r="A4" s="130"/>
       <c r="B4" s="13" t="s">
         <v>53</v>
       </c>
@@ -13946,7 +13946,7 @@
       <c r="H4" s="16"/>
     </row>
     <row r="5" spans="1:25" ht="13.8">
-      <c r="A5" s="128"/>
+      <c r="A5" s="130"/>
       <c r="B5" s="13" t="s">
         <v>55</v>
       </c>
@@ -13966,7 +13966,7 @@
       <c r="H5" s="16"/>
     </row>
     <row r="6" spans="1:25" ht="27.6">
-      <c r="A6" s="128"/>
+      <c r="A6" s="130"/>
       <c r="B6" s="13" t="s">
         <v>56</v>
       </c>
@@ -13986,7 +13986,7 @@
       <c r="H6" s="17"/>
     </row>
     <row r="7" spans="1:25" ht="27.6">
-      <c r="A7" s="128"/>
+      <c r="A7" s="130"/>
       <c r="B7" s="13" t="s">
         <v>58</v>
       </c>
@@ -14006,7 +14006,7 @@
       <c r="H7" s="16"/>
     </row>
     <row r="8" spans="1:25" ht="41.4">
-      <c r="A8" s="128"/>
+      <c r="A8" s="130"/>
       <c r="B8" s="27" t="s">
         <v>60</v>
       </c>
@@ -14026,7 +14026,7 @@
       <c r="H8" s="16"/>
     </row>
     <row r="9" spans="1:25" ht="55.2">
-      <c r="A9" s="128"/>
+      <c r="A9" s="130"/>
       <c r="B9" s="13" t="s">
         <v>61</v>
       </c>
@@ -14046,7 +14046,7 @@
       <c r="H9" s="16"/>
     </row>
     <row r="10" spans="1:25" ht="69">
-      <c r="A10" s="128"/>
+      <c r="A10" s="130"/>
       <c r="B10" s="13" t="s">
         <v>63</v>
       </c>
@@ -14066,7 +14066,7 @@
       <c r="H10" s="16"/>
     </row>
     <row r="11" spans="1:25" ht="55.2">
-      <c r="A11" s="128"/>
+      <c r="A11" s="130"/>
       <c r="B11" s="13" t="s">
         <v>66</v>
       </c>
@@ -14103,7 +14103,7 @@
       <c r="Y11" s="2"/>
     </row>
     <row r="12" spans="1:25" ht="55.2">
-      <c r="A12" s="128"/>
+      <c r="A12" s="130"/>
       <c r="B12" s="13" t="s">
         <v>67</v>
       </c>
@@ -14140,7 +14140,7 @@
       <c r="Y12" s="2"/>
     </row>
     <row r="13" spans="1:25" ht="16.8" customHeight="1">
-      <c r="A13" s="133" t="s">
+      <c r="A13" s="129" t="s">
         <v>70</v>
       </c>
       <c r="B13" s="27" t="s">
@@ -14179,7 +14179,7 @@
       <c r="Y13" s="2"/>
     </row>
     <row r="14" spans="1:25" ht="30" customHeight="1">
-      <c r="A14" s="128"/>
+      <c r="A14" s="130"/>
       <c r="B14" s="27" t="s">
         <v>71</v>
       </c>
@@ -14216,7 +14216,7 @@
       <c r="Y14" s="2"/>
     </row>
     <row r="15" spans="1:25" ht="27.6">
-      <c r="A15" s="128"/>
+      <c r="A15" s="130"/>
       <c r="B15" s="27" t="s">
         <v>424</v>
       </c>
@@ -14253,7 +14253,7 @@
       <c r="Y15" s="2"/>
     </row>
     <row r="16" spans="1:25" ht="27.6">
-      <c r="A16" s="128"/>
+      <c r="A16" s="130"/>
       <c r="B16" s="27" t="s">
         <v>426</v>
       </c>
@@ -14273,7 +14273,7 @@
       <c r="H16" s="16"/>
     </row>
     <row r="17" spans="1:8" ht="41.4">
-      <c r="A17" s="128"/>
+      <c r="A17" s="130"/>
       <c r="B17" s="27" t="s">
         <v>73</v>
       </c>
@@ -14293,7 +14293,7 @@
       <c r="H17" s="16"/>
     </row>
     <row r="18" spans="1:8" ht="41.4">
-      <c r="A18" s="128"/>
+      <c r="A18" s="130"/>
       <c r="B18" s="27" t="s">
         <v>76</v>
       </c>
@@ -14313,7 +14313,7 @@
       <c r="H18" s="16"/>
     </row>
     <row r="19" spans="1:8" ht="27.6">
-      <c r="A19" s="128"/>
+      <c r="A19" s="130"/>
       <c r="B19" s="27" t="s">
         <v>79</v>
       </c>
@@ -14333,7 +14333,7 @@
       <c r="H19" s="16"/>
     </row>
     <row r="20" spans="1:8" ht="55.2">
-      <c r="A20" s="128"/>
+      <c r="A20" s="130"/>
       <c r="B20" s="27" t="s">
         <v>81</v>
       </c>
@@ -14353,7 +14353,7 @@
       <c r="H20" s="16"/>
     </row>
     <row r="21" spans="1:8" ht="92.4">
-      <c r="A21" s="128"/>
+      <c r="A21" s="130"/>
       <c r="B21" s="27" t="s">
         <v>82</v>
       </c>
@@ -14377,7 +14377,7 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="27.6">
-      <c r="A22" s="133" t="s">
+      <c r="A22" s="129" t="s">
         <v>9</v>
       </c>
       <c r="B22" s="27" t="s">
@@ -14399,7 +14399,7 @@
       <c r="H22" s="16"/>
     </row>
     <row r="23" spans="1:8" ht="27.6">
-      <c r="A23" s="128"/>
+      <c r="A23" s="130"/>
       <c r="B23" s="13" t="s">
         <v>179</v>
       </c>
@@ -14419,7 +14419,7 @@
       <c r="H23" s="16"/>
     </row>
     <row r="24" spans="1:8" ht="27.6">
-      <c r="A24" s="128"/>
+      <c r="A24" s="130"/>
       <c r="B24" s="13" t="s">
         <v>182</v>
       </c>
@@ -14439,7 +14439,7 @@
       <c r="H24" s="17"/>
     </row>
     <row r="25" spans="1:8" ht="41.4">
-      <c r="A25" s="128"/>
+      <c r="A25" s="130"/>
       <c r="B25" s="13" t="s">
         <v>180</v>
       </c>
@@ -14463,7 +14463,7 @@
       </c>
     </row>
     <row r="26" spans="1:8" ht="52.8">
-      <c r="A26" s="128"/>
+      <c r="A26" s="130"/>
       <c r="B26" s="13" t="s">
         <v>186</v>
       </c>
@@ -14487,7 +14487,7 @@
       </c>
     </row>
     <row r="27" spans="1:8" ht="41.4">
-      <c r="A27" s="128"/>
+      <c r="A27" s="130"/>
       <c r="B27" s="13" t="s">
         <v>190</v>
       </c>
@@ -14507,7 +14507,7 @@
       <c r="H27" s="16"/>
     </row>
     <row r="28" spans="1:8" ht="41.4">
-      <c r="A28" s="128"/>
+      <c r="A28" s="130"/>
       <c r="B28" s="13" t="s">
         <v>192</v>
       </c>
@@ -14527,7 +14527,7 @@
       <c r="H28" s="16"/>
     </row>
     <row r="29" spans="1:8" ht="27.6">
-      <c r="A29" s="128"/>
+      <c r="A29" s="130"/>
       <c r="B29" s="13" t="s">
         <v>194</v>
       </c>
@@ -14547,7 +14547,7 @@
       <c r="H29" s="16"/>
     </row>
     <row r="30" spans="1:8" ht="27.6">
-      <c r="A30" s="128"/>
+      <c r="A30" s="130"/>
       <c r="B30" s="13" t="s">
         <v>196</v>
       </c>
@@ -14567,7 +14567,7 @@
       <c r="H30" s="16"/>
     </row>
     <row r="31" spans="1:8" ht="27.6">
-      <c r="A31" s="128"/>
+      <c r="A31" s="130"/>
       <c r="B31" s="13" t="s">
         <v>200</v>
       </c>
@@ -14587,7 +14587,7 @@
       <c r="H31" s="16"/>
     </row>
     <row r="32" spans="1:8" ht="52.8">
-      <c r="A32" s="128"/>
+      <c r="A32" s="130"/>
       <c r="B32" s="13" t="s">
         <v>280</v>
       </c>
@@ -14611,7 +14611,7 @@
       </c>
     </row>
     <row r="33" spans="1:8" ht="55.2">
-      <c r="A33" s="128"/>
+      <c r="A33" s="130"/>
       <c r="B33" s="13" t="s">
         <v>202</v>
       </c>
@@ -14631,7 +14631,7 @@
       <c r="H33" s="16"/>
     </row>
     <row r="34" spans="1:8" ht="41.4">
-      <c r="A34" s="128"/>
+      <c r="A34" s="130"/>
       <c r="B34" s="13" t="s">
         <v>204</v>
       </c>
@@ -14655,7 +14655,7 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="27.6">
-      <c r="A35" s="133" t="s">
+      <c r="A35" s="129" t="s">
         <v>11</v>
       </c>
       <c r="B35" s="13" t="s">
@@ -14677,7 +14677,7 @@
       <c r="H35" s="16"/>
     </row>
     <row r="36" spans="1:8" ht="13.8">
-      <c r="A36" s="128"/>
+      <c r="A36" s="130"/>
       <c r="B36" s="13" t="s">
         <v>87</v>
       </c>
@@ -14697,7 +14697,7 @@
       <c r="H36" s="16"/>
     </row>
     <row r="37" spans="1:8" ht="79.2">
-      <c r="A37" s="128"/>
+      <c r="A37" s="130"/>
       <c r="B37" s="13" t="s">
         <v>89</v>
       </c>
@@ -14721,7 +14721,7 @@
       </c>
     </row>
     <row r="38" spans="1:8" ht="76.2" customHeight="1">
-      <c r="A38" s="128"/>
+      <c r="A38" s="130"/>
       <c r="B38" s="13" t="s">
         <v>276</v>
       </c>
@@ -14745,7 +14745,7 @@
       </c>
     </row>
     <row r="39" spans="1:8" ht="55.2">
-      <c r="A39" s="128"/>
+      <c r="A39" s="130"/>
       <c r="B39" s="13" t="s">
         <v>95</v>
       </c>
@@ -14765,7 +14765,7 @@
       <c r="H39" s="16"/>
     </row>
     <row r="40" spans="1:8" ht="69">
-      <c r="A40" s="128"/>
+      <c r="A40" s="130"/>
       <c r="B40" s="13" t="s">
         <v>97</v>
       </c>
@@ -14785,7 +14785,7 @@
       <c r="H40" s="16"/>
     </row>
     <row r="41" spans="1:8" ht="79.2">
-      <c r="A41" s="128"/>
+      <c r="A41" s="130"/>
       <c r="B41" s="13" t="s">
         <v>99</v>
       </c>
@@ -14809,7 +14809,7 @@
       </c>
     </row>
     <row r="42" spans="1:8" ht="69">
-      <c r="A42" s="128"/>
+      <c r="A42" s="130"/>
       <c r="B42" s="13" t="s">
         <v>104</v>
       </c>
@@ -14829,7 +14829,7 @@
       <c r="H42" s="16"/>
     </row>
     <row r="43" spans="1:8" ht="92.4">
-      <c r="A43" s="128"/>
+      <c r="A43" s="130"/>
       <c r="B43" s="13" t="s">
         <v>105</v>
       </c>
@@ -14853,7 +14853,7 @@
       </c>
     </row>
     <row r="44" spans="1:8" ht="27.6">
-      <c r="A44" s="128"/>
+      <c r="A44" s="130"/>
       <c r="B44" s="13" t="s">
         <v>109</v>
       </c>
@@ -14873,7 +14873,7 @@
       <c r="H44" s="16"/>
     </row>
     <row r="45" spans="1:8" ht="27.6">
-      <c r="A45" s="128"/>
+      <c r="A45" s="130"/>
       <c r="B45" s="13" t="s">
         <v>112</v>
       </c>
@@ -14893,7 +14893,7 @@
       <c r="H45" s="16"/>
     </row>
     <row r="46" spans="1:8" ht="27.6">
-      <c r="A46" s="133" t="s">
+      <c r="A46" s="129" t="s">
         <v>12</v>
       </c>
       <c r="B46" s="13" t="s">
@@ -14915,7 +14915,7 @@
       <c r="H46" s="16"/>
     </row>
     <row r="47" spans="1:8" ht="27.6">
-      <c r="A47" s="128"/>
+      <c r="A47" s="130"/>
       <c r="B47" s="13" t="s">
         <v>115</v>
       </c>
@@ -14935,7 +14935,7 @@
       <c r="H47" s="16"/>
     </row>
     <row r="48" spans="1:8" ht="66">
-      <c r="A48" s="128"/>
+      <c r="A48" s="130"/>
       <c r="B48" s="13" t="s">
         <v>273</v>
       </c>
@@ -14959,7 +14959,7 @@
       </c>
     </row>
     <row r="49" spans="1:8" ht="27.6">
-      <c r="A49" s="128"/>
+      <c r="A49" s="130"/>
       <c r="B49" s="13" t="s">
         <v>117</v>
       </c>
@@ -14979,7 +14979,7 @@
       <c r="H49" s="16"/>
     </row>
     <row r="50" spans="1:8" ht="27.6">
-      <c r="A50" s="128"/>
+      <c r="A50" s="130"/>
       <c r="B50" s="13" t="s">
         <v>119</v>
       </c>
@@ -14999,7 +14999,7 @@
       <c r="H50" s="16"/>
     </row>
     <row r="51" spans="1:8" ht="27.6">
-      <c r="A51" s="128"/>
+      <c r="A51" s="130"/>
       <c r="B51" s="13" t="s">
         <v>121</v>
       </c>
@@ -15019,7 +15019,7 @@
       <c r="H51" s="16"/>
     </row>
     <row r="52" spans="1:8" ht="27.6">
-      <c r="A52" s="128"/>
+      <c r="A52" s="130"/>
       <c r="B52" s="13" t="s">
         <v>123</v>
       </c>
@@ -15039,7 +15039,7 @@
       <c r="H52" s="16"/>
     </row>
     <row r="53" spans="1:8" ht="27.6">
-      <c r="A53" s="128"/>
+      <c r="A53" s="130"/>
       <c r="B53" s="13" t="s">
         <v>125</v>
       </c>
@@ -15059,7 +15059,7 @@
       <c r="H53" s="16"/>
     </row>
     <row r="54" spans="1:8" ht="27.6">
-      <c r="A54" s="128"/>
+      <c r="A54" s="130"/>
       <c r="B54" s="13" t="s">
         <v>127</v>
       </c>
@@ -15079,7 +15079,7 @@
       <c r="H54" s="16"/>
     </row>
     <row r="55" spans="1:8" ht="41.4">
-      <c r="A55" s="128"/>
+      <c r="A55" s="130"/>
       <c r="B55" s="13" t="s">
         <v>129</v>
       </c>
@@ -15099,7 +15099,7 @@
       <c r="H55" s="16"/>
     </row>
     <row r="56" spans="1:8" ht="27.6">
-      <c r="A56" s="128"/>
+      <c r="A56" s="130"/>
       <c r="B56" s="13" t="s">
         <v>130</v>
       </c>
@@ -15119,7 +15119,7 @@
       <c r="H56" s="16"/>
     </row>
     <row r="57" spans="1:8" ht="27.6">
-      <c r="A57" s="128"/>
+      <c r="A57" s="130"/>
       <c r="B57" s="13" t="s">
         <v>132</v>
       </c>
@@ -15139,7 +15139,7 @@
       <c r="H57" s="16"/>
     </row>
     <row r="58" spans="1:8" ht="27.6">
-      <c r="A58" s="128"/>
+      <c r="A58" s="130"/>
       <c r="B58" s="13" t="s">
         <v>134</v>
       </c>
@@ -15159,7 +15159,7 @@
       <c r="H58" s="16"/>
     </row>
     <row r="59" spans="1:8" ht="41.4">
-      <c r="A59" s="128"/>
+      <c r="A59" s="130"/>
       <c r="B59" s="13" t="s">
         <v>136</v>
       </c>
@@ -15179,7 +15179,7 @@
       <c r="H59" s="16"/>
     </row>
     <row r="60" spans="1:8" ht="41.4">
-      <c r="A60" s="128"/>
+      <c r="A60" s="130"/>
       <c r="B60" s="13" t="s">
         <v>137</v>
       </c>
@@ -15199,7 +15199,7 @@
       <c r="H60" s="16"/>
     </row>
     <row r="61" spans="1:8" ht="28.8" customHeight="1">
-      <c r="A61" s="128"/>
+      <c r="A61" s="130"/>
       <c r="B61" s="13" t="s">
         <v>138</v>
       </c>
@@ -15219,7 +15219,7 @@
       <c r="H61" s="16"/>
     </row>
     <row r="62" spans="1:8" ht="27.6">
-      <c r="A62" s="128"/>
+      <c r="A62" s="130"/>
       <c r="B62" s="13" t="s">
         <v>140</v>
       </c>
@@ -15239,7 +15239,7 @@
       <c r="H62" s="16"/>
     </row>
     <row r="63" spans="1:8" ht="27.6">
-      <c r="A63" s="128"/>
+      <c r="A63" s="130"/>
       <c r="B63" s="13" t="s">
         <v>142</v>
       </c>
@@ -15259,7 +15259,7 @@
       <c r="H63" s="16"/>
     </row>
     <row r="64" spans="1:8" ht="27.6">
-      <c r="A64" s="128"/>
+      <c r="A64" s="130"/>
       <c r="B64" s="13" t="s">
         <v>144</v>
       </c>
@@ -15279,7 +15279,7 @@
       <c r="H64" s="16"/>
     </row>
     <row r="65" spans="1:14" ht="52.2" customHeight="1">
-      <c r="A65" s="128"/>
+      <c r="A65" s="130"/>
       <c r="B65" s="13" t="s">
         <v>282</v>
       </c>
@@ -15303,7 +15303,7 @@
       </c>
     </row>
     <row r="66" spans="1:14" ht="41.4">
-      <c r="A66" s="128"/>
+      <c r="A66" s="130"/>
       <c r="B66" s="13" t="s">
         <v>147</v>
       </c>
@@ -15323,7 +15323,7 @@
       <c r="H66" s="16"/>
     </row>
     <row r="67" spans="1:14" ht="27.6">
-      <c r="A67" s="128"/>
+      <c r="A67" s="130"/>
       <c r="B67" s="13" t="s">
         <v>151</v>
       </c>
@@ -15343,7 +15343,7 @@
       <c r="H67" s="16"/>
     </row>
     <row r="68" spans="1:14" ht="27.6">
-      <c r="A68" s="128"/>
+      <c r="A68" s="130"/>
       <c r="B68" s="13" t="s">
         <v>149</v>
       </c>
@@ -15363,7 +15363,7 @@
       <c r="H68" s="16"/>
     </row>
     <row r="69" spans="1:14" ht="55.2">
-      <c r="A69" s="133" t="s">
+      <c r="A69" s="129" t="s">
         <v>208</v>
       </c>
       <c r="B69" s="21" t="s">
@@ -15385,7 +15385,7 @@
       <c r="H69" s="16"/>
     </row>
     <row r="70" spans="1:14" ht="42" customHeight="1">
-      <c r="A70" s="128"/>
+      <c r="A70" s="130"/>
       <c r="B70" s="21" t="s">
         <v>211</v>
       </c>
@@ -15410,7 +15410,7 @@
       <c r="N70" s="4"/>
     </row>
     <row r="71" spans="1:14" ht="55.2" customHeight="1">
-      <c r="A71" s="128"/>
+      <c r="A71" s="130"/>
       <c r="B71" s="21" t="s">
         <v>213</v>
       </c>
@@ -15435,7 +15435,7 @@
       <c r="N71" s="4"/>
     </row>
     <row r="72" spans="1:14" ht="55.2" customHeight="1">
-      <c r="A72" s="128"/>
+      <c r="A72" s="130"/>
       <c r="B72" s="21" t="s">
         <v>215</v>
       </c>
@@ -15460,7 +15460,7 @@
       <c r="N72" s="4"/>
     </row>
     <row r="73" spans="1:14" ht="55.8" customHeight="1">
-      <c r="A73" s="128"/>
+      <c r="A73" s="130"/>
       <c r="B73" s="21" t="s">
         <v>217</v>
       </c>
@@ -15485,7 +15485,7 @@
       <c r="N73" s="4"/>
     </row>
     <row r="74" spans="1:14" ht="63.6" customHeight="1">
-      <c r="A74" s="128"/>
+      <c r="A74" s="130"/>
       <c r="B74" s="21" t="s">
         <v>219</v>
       </c>
@@ -15510,7 +15510,7 @@
       <c r="N74" s="4"/>
     </row>
     <row r="75" spans="1:14" ht="41.4" customHeight="1">
-      <c r="A75" s="128"/>
+      <c r="A75" s="130"/>
       <c r="B75" s="21" t="s">
         <v>221</v>
       </c>
@@ -15535,7 +15535,7 @@
       <c r="N75" s="4"/>
     </row>
     <row r="76" spans="1:14" ht="54.6" customHeight="1">
-      <c r="A76" s="128"/>
+      <c r="A76" s="130"/>
       <c r="B76" s="21" t="s">
         <v>223</v>
       </c>
@@ -15560,7 +15560,7 @@
       <c r="N76" s="4"/>
     </row>
     <row r="77" spans="1:14" ht="42" customHeight="1">
-      <c r="A77" s="128"/>
+      <c r="A77" s="130"/>
       <c r="B77" s="21" t="s">
         <v>225</v>
       </c>
@@ -15585,7 +15585,7 @@
       <c r="N77" s="4"/>
     </row>
     <row r="78" spans="1:14" ht="55.8" customHeight="1">
-      <c r="A78" s="128"/>
+      <c r="A78" s="130"/>
       <c r="B78" s="21" t="s">
         <v>227</v>
       </c>
@@ -15610,7 +15610,7 @@
       <c r="N78" s="4"/>
     </row>
     <row r="79" spans="1:14" ht="42.6" customHeight="1">
-      <c r="A79" s="128"/>
+      <c r="A79" s="130"/>
       <c r="B79" s="21" t="s">
         <v>229</v>
       </c>
@@ -15635,7 +15635,7 @@
       <c r="N79" s="4"/>
     </row>
     <row r="80" spans="1:14" ht="41.4" customHeight="1">
-      <c r="A80" s="128"/>
+      <c r="A80" s="130"/>
       <c r="B80" s="21" t="s">
         <v>231</v>
       </c>
@@ -15660,7 +15660,7 @@
       <c r="N80" s="4"/>
     </row>
     <row r="81" spans="1:14" ht="40.799999999999997" customHeight="1">
-      <c r="A81" s="128"/>
+      <c r="A81" s="130"/>
       <c r="B81" s="21" t="s">
         <v>233</v>
       </c>
@@ -15685,7 +15685,7 @@
       <c r="N81" s="4"/>
     </row>
     <row r="82" spans="1:14" ht="42" customHeight="1">
-      <c r="A82" s="128"/>
+      <c r="A82" s="130"/>
       <c r="B82" s="21" t="s">
         <v>235</v>
       </c>
@@ -15714,7 +15714,7 @@
       <c r="N82" s="4"/>
     </row>
     <row r="83" spans="1:14" ht="42" customHeight="1">
-      <c r="A83" s="128"/>
+      <c r="A83" s="130"/>
       <c r="B83" s="21" t="s">
         <v>239</v>
       </c>
@@ -15743,7 +15743,7 @@
       <c r="N83" s="4"/>
     </row>
     <row r="84" spans="1:14" ht="40.799999999999997" customHeight="1">
-      <c r="A84" s="128"/>
+      <c r="A84" s="130"/>
       <c r="B84" s="21" t="s">
         <v>243</v>
       </c>
@@ -15772,7 +15772,7 @@
       <c r="N84" s="4"/>
     </row>
     <row r="85" spans="1:14" ht="70.2" customHeight="1">
-      <c r="A85" s="128"/>
+      <c r="A85" s="130"/>
       <c r="B85" s="21" t="s">
         <v>245</v>
       </c>
@@ -15801,7 +15801,7 @@
       <c r="N85" s="4"/>
     </row>
     <row r="86" spans="1:14" ht="59.4" customHeight="1">
-      <c r="A86" s="128"/>
+      <c r="A86" s="130"/>
       <c r="B86" s="21" t="s">
         <v>252</v>
       </c>
@@ -15830,7 +15830,7 @@
       <c r="N86" s="4"/>
     </row>
     <row r="87" spans="1:14" ht="40.799999999999997" customHeight="1">
-      <c r="A87" s="128"/>
+      <c r="A87" s="130"/>
       <c r="B87" s="21" t="s">
         <v>255</v>
       </c>
@@ -15859,7 +15859,7 @@
       <c r="N87" s="4"/>
     </row>
     <row r="88" spans="1:14" ht="55.2" customHeight="1">
-      <c r="A88" s="128"/>
+      <c r="A88" s="130"/>
       <c r="B88" s="21" t="s">
         <v>258</v>
       </c>
@@ -15884,7 +15884,7 @@
       <c r="N88" s="4"/>
     </row>
     <row r="89" spans="1:14" ht="55.8" customHeight="1">
-      <c r="A89" s="128"/>
+      <c r="A89" s="130"/>
       <c r="B89" s="21" t="s">
         <v>260</v>
       </c>
@@ -15913,7 +15913,7 @@
       <c r="N89" s="4"/>
     </row>
     <row r="90" spans="1:14" ht="45.6" customHeight="1">
-      <c r="A90" s="128"/>
+      <c r="A90" s="130"/>
       <c r="B90" s="21" t="s">
         <v>265</v>
       </c>
@@ -15938,7 +15938,7 @@
       <c r="N90" s="4"/>
     </row>
     <row r="91" spans="1:14" ht="56.4" customHeight="1">
-      <c r="A91" s="128"/>
+      <c r="A91" s="130"/>
       <c r="B91" s="21" t="s">
         <v>269</v>
       </c>
@@ -15967,7 +15967,7 @@
       <c r="N91" s="4"/>
     </row>
     <row r="92" spans="1:14" ht="42" customHeight="1">
-      <c r="A92" s="133" t="s">
+      <c r="A92" s="129" t="s">
         <v>13</v>
       </c>
       <c r="B92" s="27" t="s">
@@ -15994,7 +15994,7 @@
       <c r="N92" s="4"/>
     </row>
     <row r="93" spans="1:14" s="63" customFormat="1" ht="27.6">
-      <c r="A93" s="128"/>
+      <c r="A93" s="130"/>
       <c r="B93" s="27" t="s">
         <v>160</v>
       </c>
@@ -16016,7 +16016,7 @@
       <c r="K93" s="64"/>
     </row>
     <row r="94" spans="1:14" ht="61.2" customHeight="1">
-      <c r="A94" s="128"/>
+      <c r="A94" s="130"/>
       <c r="B94" s="27" t="s">
         <v>586</v>
       </c>
@@ -16041,7 +16041,7 @@
       <c r="N94" s="2"/>
     </row>
     <row r="95" spans="1:14" ht="27.6">
-      <c r="A95" s="128"/>
+      <c r="A95" s="130"/>
       <c r="B95" s="27" t="s">
         <v>161</v>
       </c>
@@ -16066,7 +16066,7 @@
       <c r="N95" s="2"/>
     </row>
     <row r="96" spans="1:14" ht="27.6">
-      <c r="A96" s="128"/>
+      <c r="A96" s="130"/>
       <c r="B96" s="21" t="s">
         <v>155</v>
       </c>
@@ -16091,7 +16091,7 @@
       <c r="N96" s="2"/>
     </row>
     <row r="97" spans="1:14" ht="41.4">
-      <c r="A97" s="128"/>
+      <c r="A97" s="130"/>
       <c r="B97" s="21" t="s">
         <v>156</v>
       </c>
@@ -16116,7 +16116,7 @@
       <c r="N97" s="2"/>
     </row>
     <row r="98" spans="1:14" ht="41.4">
-      <c r="A98" s="128"/>
+      <c r="A98" s="130"/>
       <c r="B98" s="21" t="s">
         <v>158</v>
       </c>
@@ -16141,7 +16141,7 @@
       <c r="N98" s="2"/>
     </row>
     <row r="99" spans="1:14" ht="41.4">
-      <c r="A99" s="128"/>
+      <c r="A99" s="130"/>
       <c r="B99" s="27" t="s">
         <v>162</v>
       </c>
@@ -16166,7 +16166,7 @@
       <c r="N99" s="2"/>
     </row>
     <row r="100" spans="1:14" ht="41.4">
-      <c r="A100" s="128"/>
+      <c r="A100" s="130"/>
       <c r="B100" s="27" t="s">
         <v>164</v>
       </c>
@@ -16191,7 +16191,7 @@
       <c r="N100" s="2"/>
     </row>
     <row r="101" spans="1:14" ht="39" customHeight="1">
-      <c r="A101" s="128"/>
+      <c r="A101" s="130"/>
       <c r="B101" s="27" t="s">
         <v>587</v>
       </c>
@@ -16216,7 +16216,7 @@
       <c r="N101" s="2"/>
     </row>
     <row r="102" spans="1:14" ht="41.4">
-      <c r="A102" s="128"/>
+      <c r="A102" s="130"/>
       <c r="B102" s="27" t="s">
         <v>166</v>
       </c>
@@ -16241,7 +16241,7 @@
       <c r="N102" s="2"/>
     </row>
     <row r="103" spans="1:14" s="63" customFormat="1" ht="69.599999999999994" customHeight="1">
-      <c r="A103" s="128"/>
+      <c r="A103" s="130"/>
       <c r="B103" s="27" t="s">
         <v>168</v>
       </c>
@@ -16266,7 +16266,7 @@
       <c r="N103" s="65"/>
     </row>
     <row r="104" spans="1:14" ht="27.6">
-      <c r="A104" s="128"/>
+      <c r="A104" s="130"/>
       <c r="B104" s="21" t="s">
         <v>169</v>
       </c>
@@ -16291,7 +16291,7 @@
       <c r="N104" s="2"/>
     </row>
     <row r="105" spans="1:14" ht="55.2">
-      <c r="A105" s="128"/>
+      <c r="A105" s="130"/>
       <c r="B105" s="21" t="s">
         <v>171</v>
       </c>
@@ -16316,7 +16316,7 @@
       <c r="N105" s="2"/>
     </row>
     <row r="106" spans="1:14" ht="44.4" customHeight="1">
-      <c r="A106" s="128"/>
+      <c r="A106" s="130"/>
       <c r="B106" s="27" t="s">
         <v>600</v>
       </c>
@@ -16341,7 +16341,7 @@
       <c r="N106" s="2"/>
     </row>
     <row r="107" spans="1:14" ht="55.2">
-      <c r="A107" s="128"/>
+      <c r="A107" s="130"/>
       <c r="B107" s="21" t="s">
         <v>173</v>
       </c>
@@ -16366,7 +16366,7 @@
       <c r="N107" s="2"/>
     </row>
     <row r="108" spans="1:14" ht="69">
-      <c r="A108" s="128"/>
+      <c r="A108" s="130"/>
       <c r="B108" s="27" t="s">
         <v>175</v>
       </c>
@@ -16391,7 +16391,7 @@
       <c r="N108" s="2"/>
     </row>
     <row r="109" spans="1:14" ht="61.8" customHeight="1">
-      <c r="A109" s="127" t="s">
+      <c r="A109" s="136" t="s">
         <v>14</v>
       </c>
       <c r="B109" s="21" t="s">
@@ -16418,7 +16418,7 @@
       <c r="N109" s="4"/>
     </row>
     <row r="110" spans="1:14" ht="60" customHeight="1">
-      <c r="A110" s="128"/>
+      <c r="A110" s="130"/>
       <c r="B110" s="21" t="s">
         <v>288</v>
       </c>
@@ -16447,7 +16447,7 @@
       <c r="N110" s="4"/>
     </row>
     <row r="111" spans="1:14" ht="63" customHeight="1">
-      <c r="A111" s="128"/>
+      <c r="A111" s="130"/>
       <c r="B111" s="21" t="s">
         <v>292</v>
       </c>
@@ -16472,7 +16472,7 @@
       <c r="N111" s="4"/>
     </row>
     <row r="112" spans="1:14" ht="74.400000000000006" customHeight="1">
-      <c r="A112" s="128"/>
+      <c r="A112" s="130"/>
       <c r="B112" s="21" t="s">
         <v>294</v>
       </c>
@@ -16501,7 +16501,7 @@
       <c r="N112" s="4"/>
     </row>
     <row r="113" spans="1:14" ht="59.4" customHeight="1">
-      <c r="A113" s="128"/>
+      <c r="A113" s="130"/>
       <c r="B113" s="21" t="s">
         <v>299</v>
       </c>
@@ -16526,7 +16526,7 @@
       <c r="N113" s="4"/>
     </row>
     <row r="114" spans="1:14" ht="41.4">
-      <c r="A114" s="128"/>
+      <c r="A114" s="130"/>
       <c r="B114" s="21" t="s">
         <v>300</v>
       </c>
@@ -16551,7 +16551,7 @@
       <c r="N114" s="4"/>
     </row>
     <row r="115" spans="1:14" ht="40.799999999999997" customHeight="1">
-      <c r="A115" s="128"/>
+      <c r="A115" s="130"/>
       <c r="B115" s="21" t="s">
         <v>302</v>
       </c>
@@ -16576,7 +16576,7 @@
       <c r="N115" s="4"/>
     </row>
     <row r="116" spans="1:14" ht="45.6" customHeight="1">
-      <c r="A116" s="128"/>
+      <c r="A116" s="130"/>
       <c r="B116" s="21" t="s">
         <v>304</v>
       </c>
@@ -16601,7 +16601,7 @@
       <c r="N116" s="4"/>
     </row>
     <row r="117" spans="1:14" ht="44.4" customHeight="1">
-      <c r="A117" s="128"/>
+      <c r="A117" s="130"/>
       <c r="B117" s="21" t="s">
         <v>306</v>
       </c>
@@ -16626,7 +16626,7 @@
       <c r="N117" s="4"/>
     </row>
     <row r="118" spans="1:14" ht="77.400000000000006" customHeight="1">
-      <c r="A118" s="128"/>
+      <c r="A118" s="130"/>
       <c r="B118" s="21" t="s">
         <v>308</v>
       </c>
@@ -16655,7 +16655,7 @@
       <c r="N118" s="4"/>
     </row>
     <row r="119" spans="1:14" ht="65.400000000000006" customHeight="1">
-      <c r="A119" s="128"/>
+      <c r="A119" s="130"/>
       <c r="B119" s="21" t="s">
         <v>312</v>
       </c>
@@ -16680,7 +16680,7 @@
       <c r="N119" s="4"/>
     </row>
     <row r="120" spans="1:14" ht="60.6" customHeight="1">
-      <c r="A120" s="128"/>
+      <c r="A120" s="130"/>
       <c r="B120" s="21" t="s">
         <v>314</v>
       </c>
@@ -16705,7 +16705,7 @@
       <c r="N120" s="4"/>
     </row>
     <row r="121" spans="1:14" ht="40.200000000000003" customHeight="1">
-      <c r="A121" s="128"/>
+      <c r="A121" s="130"/>
       <c r="B121" s="21" t="s">
         <v>316</v>
       </c>
@@ -16730,7 +16730,7 @@
       <c r="N121" s="4"/>
     </row>
     <row r="122" spans="1:14" ht="69">
-      <c r="A122" s="128"/>
+      <c r="A122" s="130"/>
       <c r="B122" s="21" t="s">
         <v>318</v>
       </c>
@@ -16755,7 +16755,7 @@
       <c r="N122" s="4"/>
     </row>
     <row r="123" spans="1:14" ht="60" customHeight="1">
-      <c r="A123" s="128"/>
+      <c r="A123" s="130"/>
       <c r="B123" s="21" t="s">
         <v>320</v>
       </c>
@@ -16780,7 +16780,7 @@
       <c r="N123" s="4"/>
     </row>
     <row r="124" spans="1:14" ht="69">
-      <c r="A124" s="128"/>
+      <c r="A124" s="130"/>
       <c r="B124" s="21" t="s">
         <v>322</v>
       </c>
@@ -16805,7 +16805,7 @@
       <c r="N124" s="4"/>
     </row>
     <row r="125" spans="1:14" ht="67.8" customHeight="1">
-      <c r="A125" s="128"/>
+      <c r="A125" s="130"/>
       <c r="B125" s="27" t="s">
         <v>324</v>
       </c>
@@ -19804,12 +19804,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A3:A12"/>
-    <mergeCell ref="A13:A21"/>
-    <mergeCell ref="A92:A108"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="G1:G2"/>
     <mergeCell ref="A109:A125"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:C1"/>
@@ -19817,6 +19811,12 @@
     <mergeCell ref="A35:A45"/>
     <mergeCell ref="A46:A68"/>
     <mergeCell ref="A69:A91"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="A3:A12"/>
+    <mergeCell ref="A13:A21"/>
+    <mergeCell ref="A92:A108"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <phoneticPr fontId="22" type="noConversion"/>
   <conditionalFormatting sqref="D1:F1048576 C2">
@@ -19870,44 +19870,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="13.2">
-      <c r="A1" s="145" t="s">
+      <c r="A1" s="151" t="s">
         <v>368</v>
       </c>
-      <c r="B1" s="145" t="s">
+      <c r="B1" s="151" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="145" t="s">
+      <c r="C1" s="151" t="s">
         <v>367</v>
       </c>
-      <c r="D1" s="145" t="s">
+      <c r="D1" s="151" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="145" t="s">
+      <c r="E1" s="151" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="145" t="s">
+      <c r="F1" s="151" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="145" t="s">
+      <c r="G1" s="151" t="s">
         <v>835</v>
       </c>
-      <c r="H1" s="140" t="s">
+      <c r="H1" s="148" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="141"/>
-      <c r="J1" s="142"/>
-      <c r="K1" s="143" t="s">
+      <c r="I1" s="149"/>
+      <c r="J1" s="150"/>
+      <c r="K1" s="140" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="27.6">
-      <c r="A2" s="144"/>
-      <c r="B2" s="144"/>
-      <c r="C2" s="144"/>
-      <c r="D2" s="144"/>
-      <c r="E2" s="144"/>
-      <c r="F2" s="144"/>
-      <c r="G2" s="144"/>
+      <c r="A2" s="146"/>
+      <c r="B2" s="146"/>
+      <c r="C2" s="146"/>
+      <c r="D2" s="146"/>
+      <c r="E2" s="146"/>
+      <c r="F2" s="146"/>
+      <c r="G2" s="146"/>
       <c r="H2" s="36" t="s">
         <v>21</v>
       </c>
@@ -19917,10 +19917,10 @@
       <c r="J2" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="144"/>
+      <c r="K2" s="146"/>
     </row>
     <row r="3" spans="1:11" ht="18" customHeight="1">
-      <c r="A3" s="149" t="s">
+      <c r="A3" s="144" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="38" t="s">
@@ -19953,7 +19953,7 @@
       <c r="K3" s="41"/>
     </row>
     <row r="4" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A4" s="150"/>
+      <c r="A4" s="145"/>
       <c r="B4" s="38" t="s">
         <v>336</v>
       </c>
@@ -19984,7 +19984,7 @@
       <c r="K4" s="41"/>
     </row>
     <row r="5" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A5" s="150"/>
+      <c r="A5" s="145"/>
       <c r="B5" s="38" t="s">
         <v>337</v>
       </c>
@@ -20015,7 +20015,7 @@
       <c r="K5" s="41"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A6" s="150"/>
+      <c r="A6" s="145"/>
       <c r="B6" s="38" t="s">
         <v>338</v>
       </c>
@@ -20046,7 +20046,7 @@
       <c r="K6" s="41"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A7" s="150"/>
+      <c r="A7" s="145"/>
       <c r="B7" s="38" t="s">
         <v>339</v>
       </c>
@@ -20077,7 +20077,7 @@
       <c r="K7" s="41"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A8" s="150"/>
+      <c r="A8" s="145"/>
       <c r="B8" s="38" t="s">
         <v>340</v>
       </c>
@@ -20108,7 +20108,7 @@
       <c r="K8" s="41"/>
     </row>
     <row r="9" spans="1:11" ht="15" customHeight="1">
-      <c r="A9" s="144"/>
+      <c r="A9" s="146"/>
       <c r="B9" s="38" t="s">
         <v>341</v>
       </c>
@@ -20139,7 +20139,7 @@
       <c r="K9" s="41"/>
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A10" s="149" t="s">
+      <c r="A10" s="144" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="38" t="s">
@@ -20172,7 +20172,7 @@
       <c r="K10" s="41"/>
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A11" s="150"/>
+      <c r="A11" s="145"/>
       <c r="B11" s="38" t="s">
         <v>343</v>
       </c>
@@ -20203,7 +20203,7 @@
       <c r="K11" s="41"/>
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A12" s="150"/>
+      <c r="A12" s="145"/>
       <c r="B12" s="38" t="s">
         <v>344</v>
       </c>
@@ -20234,7 +20234,7 @@
       <c r="K12" s="41"/>
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A13" s="150"/>
+      <c r="A13" s="145"/>
       <c r="B13" s="38" t="s">
         <v>345</v>
       </c>
@@ -20265,7 +20265,7 @@
       <c r="K13" s="41"/>
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A14" s="150"/>
+      <c r="A14" s="145"/>
       <c r="B14" s="38" t="s">
         <v>346</v>
       </c>
@@ -20296,7 +20296,7 @@
       <c r="K14" s="41"/>
     </row>
     <row r="15" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A15" s="150"/>
+      <c r="A15" s="145"/>
       <c r="B15" s="38" t="s">
         <v>347</v>
       </c>
@@ -20327,7 +20327,7 @@
       <c r="K15" s="41"/>
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A16" s="150"/>
+      <c r="A16" s="145"/>
       <c r="B16" s="38" t="s">
         <v>348</v>
       </c>
@@ -20358,7 +20358,7 @@
       <c r="K16" s="41"/>
     </row>
     <row r="17" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A17" s="150"/>
+      <c r="A17" s="145"/>
       <c r="B17" s="38" t="s">
         <v>349</v>
       </c>
@@ -20391,7 +20391,7 @@
       </c>
     </row>
     <row r="18" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A18" s="150"/>
+      <c r="A18" s="145"/>
       <c r="B18" s="38" t="s">
         <v>436</v>
       </c>
@@ -20422,7 +20422,7 @@
       <c r="K18" s="41"/>
     </row>
     <row r="19" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A19" s="144"/>
+      <c r="A19" s="146"/>
       <c r="B19" s="38" t="s">
         <v>437</v>
       </c>
@@ -20453,7 +20453,7 @@
       <c r="K19" s="41"/>
     </row>
     <row r="20" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A20" s="149" t="s">
+      <c r="A20" s="144" t="s">
         <v>9</v>
       </c>
       <c r="B20" s="38" t="s">
@@ -20486,7 +20486,7 @@
       <c r="K20" s="41"/>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A21" s="150"/>
+      <c r="A21" s="145"/>
       <c r="B21" s="38" t="s">
         <v>351</v>
       </c>
@@ -20517,7 +20517,7 @@
       <c r="K21" s="41"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A22" s="150"/>
+      <c r="A22" s="145"/>
       <c r="B22" s="38" t="s">
         <v>352</v>
       </c>
@@ -20550,7 +20550,7 @@
       </c>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A23" s="150"/>
+      <c r="A23" s="145"/>
       <c r="B23" s="38" t="s">
         <v>353</v>
       </c>
@@ -20583,7 +20583,7 @@
       </c>
     </row>
     <row r="24" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A24" s="150"/>
+      <c r="A24" s="145"/>
       <c r="B24" s="38" t="s">
         <v>446</v>
       </c>
@@ -20614,7 +20614,7 @@
       <c r="K24" s="41"/>
     </row>
     <row r="25" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A25" s="150"/>
+      <c r="A25" s="145"/>
       <c r="B25" s="38" t="s">
         <v>354</v>
       </c>
@@ -20645,7 +20645,7 @@
       <c r="K25" s="41"/>
     </row>
     <row r="26" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A26" s="150"/>
+      <c r="A26" s="145"/>
       <c r="B26" s="38" t="s">
         <v>355</v>
       </c>
@@ -20676,7 +20676,7 @@
       <c r="K26" s="41"/>
     </row>
     <row r="27" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A27" s="150"/>
+      <c r="A27" s="145"/>
       <c r="B27" s="38" t="s">
         <v>356</v>
       </c>
@@ -20709,7 +20709,7 @@
       </c>
     </row>
     <row r="28" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A28" s="150"/>
+      <c r="A28" s="145"/>
       <c r="B28" s="38" t="s">
         <v>357</v>
       </c>
@@ -20742,7 +20742,7 @@
       </c>
     </row>
     <row r="29" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A29" s="150"/>
+      <c r="A29" s="145"/>
       <c r="B29" s="38" t="s">
         <v>389</v>
       </c>
@@ -20773,7 +20773,7 @@
       <c r="K29" s="41"/>
     </row>
     <row r="30" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A30" s="150"/>
+      <c r="A30" s="145"/>
       <c r="B30" s="38" t="s">
         <v>390</v>
       </c>
@@ -20804,7 +20804,7 @@
       <c r="K30" s="41"/>
     </row>
     <row r="31" spans="1:11" ht="85.8" customHeight="1">
-      <c r="A31" s="151" t="s">
+      <c r="A31" s="147" t="s">
         <v>11</v>
       </c>
       <c r="B31" s="38" t="s">
@@ -20837,7 +20837,7 @@
       <c r="K31" s="41"/>
     </row>
     <row r="32" spans="1:11" ht="55.2">
-      <c r="A32" s="150"/>
+      <c r="A32" s="145"/>
       <c r="B32" s="38" t="s">
         <v>451</v>
       </c>
@@ -20870,7 +20870,7 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="82.8">
-      <c r="A33" s="150"/>
+      <c r="A33" s="145"/>
       <c r="B33" s="38" t="s">
         <v>452</v>
       </c>
@@ -20903,7 +20903,7 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="96.6">
-      <c r="A34" s="150"/>
+      <c r="A34" s="145"/>
       <c r="B34" s="38" t="s">
         <v>453</v>
       </c>
@@ -20934,7 +20934,7 @@
       <c r="K34" s="41"/>
     </row>
     <row r="35" spans="1:11" ht="82.8">
-      <c r="A35" s="150"/>
+      <c r="A35" s="145"/>
       <c r="B35" s="38" t="s">
         <v>454</v>
       </c>
@@ -20967,7 +20967,7 @@
       </c>
     </row>
     <row r="36" spans="1:11" ht="69">
-      <c r="A36" s="150"/>
+      <c r="A36" s="145"/>
       <c r="B36" s="38" t="s">
         <v>455</v>
       </c>
@@ -20998,7 +20998,7 @@
       <c r="K36" s="41"/>
     </row>
     <row r="37" spans="1:11" ht="57" customHeight="1">
-      <c r="A37" s="150"/>
+      <c r="A37" s="145"/>
       <c r="B37" s="38" t="s">
         <v>456</v>
       </c>
@@ -21031,7 +21031,7 @@
       </c>
     </row>
     <row r="38" spans="1:11" ht="72" customHeight="1">
-      <c r="A38" s="150"/>
+      <c r="A38" s="145"/>
       <c r="B38" s="38" t="s">
         <v>473</v>
       </c>
@@ -21062,7 +21062,7 @@
       <c r="K38" s="41"/>
     </row>
     <row r="39" spans="1:11" ht="92.4">
-      <c r="A39" s="149" t="s">
+      <c r="A39" s="144" t="s">
         <v>12</v>
       </c>
       <c r="B39" s="38" t="s">
@@ -21095,7 +21095,7 @@
       <c r="K39" s="41"/>
     </row>
     <row r="40" spans="1:11" ht="110.4">
-      <c r="A40" s="150"/>
+      <c r="A40" s="145"/>
       <c r="B40" s="38" t="s">
         <v>482</v>
       </c>
@@ -21126,7 +21126,7 @@
       <c r="K40" s="41"/>
     </row>
     <row r="41" spans="1:11" ht="57.6" customHeight="1">
-      <c r="A41" s="150"/>
+      <c r="A41" s="145"/>
       <c r="B41" s="38" t="s">
         <v>483</v>
       </c>
@@ -21157,7 +21157,7 @@
       <c r="K41" s="41"/>
     </row>
     <row r="42" spans="1:11" ht="61.2" customHeight="1">
-      <c r="A42" s="150"/>
+      <c r="A42" s="145"/>
       <c r="B42" s="38" t="s">
         <v>484</v>
       </c>
@@ -21188,7 +21188,7 @@
       <c r="K42" s="41"/>
     </row>
     <row r="43" spans="1:11" ht="69" customHeight="1">
-      <c r="A43" s="150"/>
+      <c r="A43" s="145"/>
       <c r="B43" s="38" t="s">
         <v>485</v>
       </c>
@@ -21219,7 +21219,7 @@
       <c r="K43" s="41"/>
     </row>
     <row r="44" spans="1:11" ht="73.8" customHeight="1">
-      <c r="A44" s="150"/>
+      <c r="A44" s="145"/>
       <c r="B44" s="38" t="s">
         <v>486</v>
       </c>
@@ -21250,7 +21250,7 @@
       <c r="K44" s="41"/>
     </row>
     <row r="45" spans="1:11" ht="85.2" customHeight="1">
-      <c r="A45" s="150"/>
+      <c r="A45" s="145"/>
       <c r="B45" s="38" t="s">
         <v>487</v>
       </c>
@@ -21281,7 +21281,7 @@
       <c r="K45" s="41"/>
     </row>
     <row r="46" spans="1:11" ht="70.8" customHeight="1">
-      <c r="A46" s="150"/>
+      <c r="A46" s="145"/>
       <c r="B46" s="38" t="s">
         <v>488</v>
       </c>
@@ -21314,7 +21314,7 @@
       </c>
     </row>
     <row r="47" spans="1:11" ht="99" customHeight="1">
-      <c r="A47" s="150"/>
+      <c r="A47" s="145"/>
       <c r="B47" s="38" t="s">
         <v>510</v>
       </c>
@@ -21347,7 +21347,7 @@
       </c>
     </row>
     <row r="48" spans="1:11" ht="92.4" customHeight="1">
-      <c r="A48" s="150"/>
+      <c r="A48" s="145"/>
       <c r="B48" s="38" t="s">
         <v>513</v>
       </c>
@@ -21378,7 +21378,7 @@
       <c r="K48" s="41"/>
     </row>
     <row r="49" spans="1:11" ht="72" customHeight="1">
-      <c r="A49" s="144"/>
+      <c r="A49" s="146"/>
       <c r="B49" s="38" t="s">
         <v>514</v>
       </c>
@@ -21409,7 +21409,7 @@
       <c r="K49" s="41"/>
     </row>
     <row r="50" spans="1:11" ht="82.8">
-      <c r="A50" s="149" t="s">
+      <c r="A50" s="144" t="s">
         <v>208</v>
       </c>
       <c r="B50" s="38" t="s">
@@ -21442,7 +21442,7 @@
       <c r="K50" s="41"/>
     </row>
     <row r="51" spans="1:11" ht="112.8" customHeight="1">
-      <c r="A51" s="150"/>
+      <c r="A51" s="145"/>
       <c r="B51" s="38" t="s">
         <v>522</v>
       </c>
@@ -21473,7 +21473,7 @@
       <c r="K51" s="41"/>
     </row>
     <row r="52" spans="1:11" ht="96.6">
-      <c r="A52" s="150"/>
+      <c r="A52" s="145"/>
       <c r="B52" s="38" t="s">
         <v>523</v>
       </c>
@@ -21504,7 +21504,7 @@
       <c r="K52" s="41"/>
     </row>
     <row r="53" spans="1:11" ht="82.2" customHeight="1">
-      <c r="A53" s="150"/>
+      <c r="A53" s="145"/>
       <c r="B53" s="38" t="s">
         <v>524</v>
       </c>
@@ -21535,7 +21535,7 @@
       <c r="K53" s="44"/>
     </row>
     <row r="54" spans="1:11" ht="82.8">
-      <c r="A54" s="150"/>
+      <c r="A54" s="145"/>
       <c r="B54" s="38" t="s">
         <v>525</v>
       </c>
@@ -21568,7 +21568,7 @@
       </c>
     </row>
     <row r="55" spans="1:11" ht="55.2">
-      <c r="A55" s="150"/>
+      <c r="A55" s="145"/>
       <c r="B55" s="38" t="s">
         <v>526</v>
       </c>
@@ -21601,7 +21601,7 @@
       </c>
     </row>
     <row r="56" spans="1:11" ht="41.4">
-      <c r="A56" s="150"/>
+      <c r="A56" s="145"/>
       <c r="B56" s="38" t="s">
         <v>527</v>
       </c>
@@ -21634,7 +21634,7 @@
       </c>
     </row>
     <row r="57" spans="1:11" ht="55.8">
-      <c r="A57" s="150"/>
+      <c r="A57" s="145"/>
       <c r="B57" s="38" t="s">
         <v>528</v>
       </c>
@@ -21667,7 +21667,7 @@
       </c>
     </row>
     <row r="58" spans="1:11" ht="82.8">
-      <c r="A58" s="150"/>
+      <c r="A58" s="145"/>
       <c r="B58" s="38" t="s">
         <v>529</v>
       </c>
@@ -21698,7 +21698,7 @@
       <c r="K58" s="41"/>
     </row>
     <row r="59" spans="1:11" ht="82.8">
-      <c r="A59" s="150"/>
+      <c r="A59" s="145"/>
       <c r="B59" s="38" t="s">
         <v>530</v>
       </c>
@@ -21731,7 +21731,7 @@
       </c>
     </row>
     <row r="60" spans="1:11" ht="55.2">
-      <c r="A60" s="150"/>
+      <c r="A60" s="145"/>
       <c r="B60" s="38" t="s">
         <v>531</v>
       </c>
@@ -21762,7 +21762,7 @@
       <c r="K60" s="41"/>
     </row>
     <row r="61" spans="1:11" ht="69">
-      <c r="A61" s="150"/>
+      <c r="A61" s="145"/>
       <c r="B61" s="38" t="s">
         <v>532</v>
       </c>
@@ -21795,7 +21795,7 @@
       </c>
     </row>
     <row r="62" spans="1:11" ht="69.599999999999994">
-      <c r="A62" s="150"/>
+      <c r="A62" s="145"/>
       <c r="B62" s="38" t="s">
         <v>533</v>
       </c>
@@ -21826,7 +21826,7 @@
       <c r="K62" s="44"/>
     </row>
     <row r="63" spans="1:11" ht="117.6" customHeight="1">
-      <c r="A63" s="150"/>
+      <c r="A63" s="145"/>
       <c r="B63" s="38" t="s">
         <v>534</v>
       </c>
@@ -21857,7 +21857,7 @@
       <c r="K63" s="41"/>
     </row>
     <row r="64" spans="1:11" ht="83.4">
-      <c r="A64" s="149" t="s">
+      <c r="A64" s="144" t="s">
         <v>13</v>
       </c>
       <c r="B64" s="38" t="s">
@@ -21890,7 +21890,7 @@
       <c r="K64" s="41"/>
     </row>
     <row r="65" spans="1:27" ht="69.599999999999994">
-      <c r="A65" s="150"/>
+      <c r="A65" s="145"/>
       <c r="B65" s="38" t="s">
         <v>574</v>
       </c>
@@ -21937,7 +21937,7 @@
       <c r="AA65" s="2"/>
     </row>
     <row r="66" spans="1:27" ht="83.4">
-      <c r="A66" s="150"/>
+      <c r="A66" s="145"/>
       <c r="B66" s="38" t="s">
         <v>575</v>
       </c>
@@ -21984,7 +21984,7 @@
       <c r="AA66" s="2"/>
     </row>
     <row r="67" spans="1:27" ht="104.4" customHeight="1">
-      <c r="A67" s="150"/>
+      <c r="A67" s="145"/>
       <c r="B67" s="38" t="s">
         <v>576</v>
       </c>
@@ -22031,7 +22031,7 @@
       <c r="AA67" s="2"/>
     </row>
     <row r="68" spans="1:27" ht="75" customHeight="1">
-      <c r="A68" s="150"/>
+      <c r="A68" s="145"/>
       <c r="B68" s="38" t="s">
         <v>577</v>
       </c>
@@ -22078,7 +22078,7 @@
       <c r="AA68" s="2"/>
     </row>
     <row r="69" spans="1:27" ht="83.4">
-      <c r="A69" s="150"/>
+      <c r="A69" s="145"/>
       <c r="B69" s="38" t="s">
         <v>578</v>
       </c>
@@ -22125,7 +22125,7 @@
       <c r="AA69" s="2"/>
     </row>
     <row r="70" spans="1:27" ht="42">
-      <c r="A70" s="150"/>
+      <c r="A70" s="145"/>
       <c r="B70" s="38" t="s">
         <v>579</v>
       </c>
@@ -22172,7 +22172,7 @@
       <c r="AA70" s="2"/>
     </row>
     <row r="71" spans="1:27" ht="78">
-      <c r="A71" s="150"/>
+      <c r="A71" s="145"/>
       <c r="B71" s="38" t="s">
         <v>580</v>
       </c>
@@ -22219,7 +22219,7 @@
       <c r="AA71" s="2"/>
     </row>
     <row r="72" spans="1:27" ht="78">
-      <c r="A72" s="150"/>
+      <c r="A72" s="145"/>
       <c r="B72" s="38" t="s">
         <v>581</v>
       </c>
@@ -22250,7 +22250,7 @@
       <c r="K72" s="41"/>
     </row>
     <row r="73" spans="1:27" ht="94.8" customHeight="1">
-      <c r="A73" s="143" t="s">
+      <c r="A73" s="140" t="s">
         <v>14</v>
       </c>
       <c r="B73" s="38" t="s">
@@ -22283,7 +22283,7 @@
       <c r="K73" s="41"/>
     </row>
     <row r="74" spans="1:27" ht="75">
-      <c r="A74" s="146"/>
+      <c r="A74" s="141"/>
       <c r="B74" s="38" t="s">
         <v>621</v>
       </c>
@@ -22316,7 +22316,7 @@
       </c>
     </row>
     <row r="75" spans="1:27" ht="75">
-      <c r="A75" s="146"/>
+      <c r="A75" s="141"/>
       <c r="B75" s="38" t="s">
         <v>622</v>
       </c>
@@ -22349,7 +22349,7 @@
       </c>
     </row>
     <row r="76" spans="1:27" ht="79.2" customHeight="1">
-      <c r="A76" s="146"/>
+      <c r="A76" s="141"/>
       <c r="B76" s="38" t="s">
         <v>623</v>
       </c>
@@ -22380,7 +22380,7 @@
       <c r="K76" s="41"/>
     </row>
     <row r="77" spans="1:27" ht="69" customHeight="1">
-      <c r="A77" s="146"/>
+      <c r="A77" s="141"/>
       <c r="B77" s="38" t="s">
         <v>633</v>
       </c>
@@ -22411,7 +22411,7 @@
       <c r="K77" s="41"/>
     </row>
     <row r="78" spans="1:27" ht="69" customHeight="1">
-      <c r="A78" s="146"/>
+      <c r="A78" s="141"/>
       <c r="B78" s="38" t="s">
         <v>637</v>
       </c>
@@ -22442,7 +22442,7 @@
       <c r="K78" s="41"/>
     </row>
     <row r="79" spans="1:27" ht="69" customHeight="1">
-      <c r="A79" s="146"/>
+      <c r="A79" s="141"/>
       <c r="B79" s="38" t="s">
         <v>641</v>
       </c>
@@ -22475,7 +22475,7 @@
       </c>
     </row>
     <row r="80" spans="1:27" ht="75" customHeight="1">
-      <c r="A80" s="146"/>
+      <c r="A80" s="141"/>
       <c r="B80" s="38" t="s">
         <v>645</v>
       </c>
@@ -22506,7 +22506,7 @@
       <c r="K80" s="41"/>
     </row>
     <row r="81" spans="1:11" ht="93" customHeight="1">
-      <c r="A81" s="146"/>
+      <c r="A81" s="141"/>
       <c r="B81" s="38" t="s">
         <v>649</v>
       </c>
@@ -22537,7 +22537,7 @@
       <c r="K81" s="41"/>
     </row>
     <row r="82" spans="1:11" ht="112.8" customHeight="1">
-      <c r="A82" s="146"/>
+      <c r="A82" s="141"/>
       <c r="B82" s="38" t="s">
         <v>653</v>
       </c>
@@ -22568,7 +22568,7 @@
       <c r="K82" s="41"/>
     </row>
     <row r="83" spans="1:11" ht="110.4" customHeight="1">
-      <c r="A83" s="146"/>
+      <c r="A83" s="141"/>
       <c r="B83" s="38" t="s">
         <v>657</v>
       </c>
@@ -22576,7 +22576,7 @@
         <v>658</v>
       </c>
       <c r="D83" s="43" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E83" s="51" t="s">
         <v>659</v>
@@ -22599,7 +22599,7 @@
       <c r="K83" s="41"/>
     </row>
     <row r="84" spans="1:11" ht="109.2" customHeight="1">
-      <c r="A84" s="146"/>
+      <c r="A84" s="141"/>
       <c r="B84" s="38" t="s">
         <v>661</v>
       </c>
@@ -22630,7 +22630,7 @@
       <c r="K84" s="41"/>
     </row>
     <row r="85" spans="1:11" ht="67.8" customHeight="1">
-      <c r="A85" s="146"/>
+      <c r="A85" s="141"/>
       <c r="B85" s="38" t="s">
         <v>665</v>
       </c>
@@ -22671,8 +22671,8 @@
     </row>
     <row r="88" spans="1:11" ht="13.2">
       <c r="A88" s="37"/>
-      <c r="B88" s="147"/>
-      <c r="C88" s="148"/>
+      <c r="B88" s="142"/>
+      <c r="C88" s="143"/>
       <c r="D88" s="10"/>
     </row>
     <row r="89" spans="1:11" ht="13.2">
@@ -25630,6 +25630,15 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
     <mergeCell ref="A73:A85"/>
     <mergeCell ref="B88:C88"/>
     <mergeCell ref="A3:A9"/>
@@ -25639,15 +25648,6 @@
     <mergeCell ref="A39:A49"/>
     <mergeCell ref="A50:A63"/>
     <mergeCell ref="A64:A72"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="K1:K2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
   </mergeCells>
   <phoneticPr fontId="22" type="noConversion"/>
   <conditionalFormatting sqref="D1:D1048576">
@@ -25709,26 +25709,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="14.4" customHeight="1">
-      <c r="A1" s="154" t="s">
+      <c r="A1" s="152" t="s">
         <v>35</v>
       </c>
       <c r="B1" s="71"/>
-      <c r="C1" s="154" t="s">
+      <c r="C1" s="152" t="s">
         <v>36</v>
       </c>
       <c r="D1" s="162" t="s">
         <v>704</v>
       </c>
-      <c r="E1" s="154" t="s">
+      <c r="E1" s="152" t="s">
         <v>38</v>
       </c>
-      <c r="F1" s="154" t="s">
+      <c r="F1" s="152" t="s">
         <v>39</v>
       </c>
-      <c r="G1" s="154" t="s">
+      <c r="G1" s="152" t="s">
         <v>40</v>
       </c>
-      <c r="H1" s="154" t="s">
+      <c r="H1" s="152" t="s">
         <v>41</v>
       </c>
       <c r="I1" s="156" t="s">
@@ -25738,16 +25738,16 @@
       <c r="K1" s="157"/>
     </row>
     <row r="2" spans="1:11" ht="42">
-      <c r="A2" s="155"/>
+      <c r="A2" s="153"/>
       <c r="B2" s="71" t="s">
         <v>705</v>
       </c>
-      <c r="C2" s="155"/>
+      <c r="C2" s="153"/>
       <c r="D2" s="163"/>
-      <c r="E2" s="155"/>
-      <c r="F2" s="155"/>
-      <c r="G2" s="155"/>
-      <c r="H2" s="155"/>
+      <c r="E2" s="153"/>
+      <c r="F2" s="153"/>
+      <c r="G2" s="153"/>
+      <c r="H2" s="153"/>
       <c r="I2" s="73" t="s">
         <v>46</v>
       </c>
@@ -26426,20 +26426,20 @@
       <c r="H22" s="160" t="s">
         <v>45</v>
       </c>
-      <c r="I22" s="152" t="s">
+      <c r="I22" s="154" t="s">
         <v>42</v>
       </c>
-      <c r="J22" s="153"/>
-      <c r="K22" s="153"/>
+      <c r="J22" s="155"/>
+      <c r="K22" s="155"/>
     </row>
     <row r="23" spans="1:11" ht="41.4">
-      <c r="A23" s="155"/>
+      <c r="A23" s="153"/>
       <c r="B23" s="89"/>
-      <c r="C23" s="155"/>
-      <c r="D23" s="155"/>
-      <c r="E23" s="155"/>
-      <c r="F23" s="155"/>
-      <c r="G23" s="155"/>
+      <c r="C23" s="153"/>
+      <c r="D23" s="153"/>
+      <c r="E23" s="153"/>
+      <c r="F23" s="153"/>
+      <c r="G23" s="153"/>
       <c r="H23" s="161"/>
       <c r="I23" s="90" t="s">
         <v>46</v>
@@ -27611,6 +27611,7 @@
     <row r="1009" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="F1:F2"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="I22:K22"/>
     <mergeCell ref="H1:H2"/>
@@ -27627,7 +27628,6 @@
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
   </mergeCells>
   <conditionalFormatting sqref="D1:D1048576">
     <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="Minor">

</xml_diff>